<commit_message>
Formalize IES definitions into restriction axioms, fix CCOM/QUDT definitions gap, rewrite FINDINGS.md
- Added 4 owl:Restriction axioms to ies.ttl (Account Holder, Money Transfer,
  Responsible Actor State, Radio Mast), derived from IES's own declared
  domain/property/range triples and matching BFO's allValuesFrom style.
  This produces 76 structural candidates against BFO where there were
  previously zero, since IES had no restrictions at all.
- Fixed augment_w_definitions.ipynb to follow ccom.ttl's owl:imports when
  looking up definitions, since the matched CCOM-side classes are actually
  defined in the imported Common Core Ontologies file, not locally.
- Rewrote FINDINGS.md with real content (previous commit accidentally
  committed it empty) covering all three pairs and why no equivalence was
  asserted in any of them.
</commit_message>
<xml_diff>
--- a/projects/project-3/assignment/src/data/ies-axioms.xlsx
+++ b/projects/project-3/assignment/src/data/ies-axioms.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SubClassOf: Responsible Actor State</t>
+          <t>SubClassOf: Responsible Actor State | SubClassOf: holds Account only Account</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>SubClassOf: Business Event | SubClassOf: Trade Event</t>
+          <t>SubClassOf: Business Event | SubClassOf: Trade Event | SubClassOf: transfer Value only Amount Of Money</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>SubClassOf: Device | SubClassOf: System State</t>
+          <t>SubClassOf: Device | SubClassOf: System State | SubClassOf: radio Coverage only Radio Coverage Area</t>
         </is>
       </c>
     </row>
@@ -7190,7 +7190,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>SubClassOf: Actor State</t>
+          <t>SubClassOf: Actor State | SubClassOf: works For only Responsible Actor</t>
         </is>
       </c>
     </row>

</xml_diff>